<commit_message>
feat(server): serve part prices from the datasheet, drop the old catalog reader
부품 카탈로그의 조회 키를 part_id 에서 part_category 로 옮긴다. 데이터시트가
부품 마스터가 되면서 Mock Part ID·Group ID·Source ID 가 사라졌고, 남은 축이
production.parts.part_category 와 시트의 '부품 타입' 이다. 둘은 같은 값이어야 한다.

datasheet.py 를 새로 둔다. 전에는 XLSX 파서가 generate_defect_reports.py 안에만
있었고 HTTP 서버는 DB 만 봤다. 가격을 API 로 내보내려면 서버도 시트를 읽어야 해서
파서를 한 곳으로 모은다. queries.py 는 DB 전용으로 두고 합치는 일은 server.py
핸들러가 한다. 서버 런타임에 openpyxl 을 넣지 않으므로 stdlib 로만 읽고, 파일
mtime 이 바뀔 때만 다시 읽어 시트 수정이 재시작 없이 반영된다.

GET /parts/{part_id} 가 후보 3종을, requirements 가 보드당 원가를 함께 낸다.
단가는 시트에, 보드당 수량은 DB 에 있어 한쪽만으로는 원가가 나오지 않는다.
후보가 여럿이라 단가가 하나로 정해지지 않으므로 selected(= part_name 과 MPN 이
같은 후보) 와 min/max 를 같이 준다. 데이터시트를 못 읽어도 DB 응답은 살린다.

대책서 「판단자료 D」 는 대체 판정 8열에서 가격 6열로 바꾼다. 상호호환 상태·필수
재검증·불량 소견은 원본 열이 없어졌다. 부품 교체 여부 판정이 자동에서 담당자
몫으로 넘어간다.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164Nd2RQ1pjrz6BPDTL62s5
</commit_message>
<xml_diff>
--- a/MAIN_SERVER/templates/불량대책서_샘플_종결본.xlsx
+++ b/MAIN_SERVER/templates/불량대책서_샘플_종결본.xlsx
@@ -281,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -409,6 +409,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -887,7 +893,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>CAP  (C-001 · MLCC)</t>
+          <t>CAP  (MLCC)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1530,7 +1536,7 @@
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="27" t="inlineStr">
         <is>
-          <t>defect_report.alert_evidence 스냅샷 · 문서번호 QA-CAP-CRACK-20260819-001 · 수정 금지</t>
+          <t>production.unit_defects 확정 기록 · 문서번호 QA-CAP-CRACK-20260819-001 · 수정 금지</t>
         </is>
       </c>
     </row>
@@ -2309,7 +2315,7 @@
     <row r="28" ht="14" customHeight="1">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>datastation_part_checklist · part_catalog.quality_checklists.category = part_groups.category_label · 이 범주에서 무엇을 확인해야 하는지</t>
+          <t>데이터시트 Checklist 시트 · 범주 = part_groups.category_label · 이 범주에서 무엇을 확인해야 하는지</t>
         </is>
       </c>
     </row>
@@ -2423,17 +2429,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="29" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -2453,200 +2457,160 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>동일 정격만으로 drop-in 판단 금지 · 「필수 재검증」을 모두 통과하고 변경 승인이 완료된 뒤에만 적용한다.</t>
+          <t>같은 부품 타입이라는 것 외에 검증된 것은 없다 · 동일 정격만으로 drop-in 판단 금지 · 핀/패키지/정격/열/수명 재검증과 변경 승인을 거친 뒤에만 적용한다.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="23" t="inlineStr">
         <is>
-          <t>조회 시각 2026-08-19 09:00:00   ·   데이터시트 semiconductor_assembly_quality_datasheet_2026-08-18.xlsx (기준일 2026-08-18)   ·   Group ID C-001 (MLCC)   ·   후보 2종</t>
+          <t>조회 시각 2026-08-19 09:00:00   ·   데이터시트 semiconductor_assembly_quality_datasheet_2026-08-18.xlsx (기준일 2026-08-18)   ·   부품 타입 MLCC   ·   후보 3종   ·   단가 $0.09 ~ $0.15   ·   현재 선정 $0.15</t>
         </is>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>역할</t>
+          <t>제조사 / P/N</t>
         </is>
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>대체코드</t>
+          <t>핵심 정격</t>
         </is>
       </c>
       <c r="C6" s="29" t="inlineStr">
         <is>
-          <t>제조사 / P/N</t>
+          <t>공급사</t>
         </is>
       </c>
       <c r="D6" s="29" t="inlineStr">
         <is>
-          <t>핵심 사양·용도</t>
+          <t>단가</t>
         </is>
       </c>
       <c r="E6" s="29" t="inlineStr">
         <is>
-          <t>상호호환 상태</t>
+          <t>가격 기준 수량</t>
         </is>
       </c>
       <c r="F6" s="29" t="inlineStr">
         <is>
-          <t>필수 재검증</t>
-        </is>
-      </c>
-      <c r="G6" s="29" t="inlineStr">
-        <is>
-          <t>CRACK 관련 소견</t>
-        </is>
-      </c>
-      <c r="H6" s="29" t="inlineStr">
-        <is>
-          <t>Source · 확인일</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
+          <t>가격 확인일</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="54" customHeight="1">
       <c r="A7" s="42" t="inlineStr">
         <is>
-          <t>주품목</t>
+          <t>Contoso CX-0603X7R104K100</t>
         </is>
       </c>
       <c r="B7" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.10µF ±10% 100V X7R 0603</t>
         </is>
       </c>
       <c r="C7" s="42" t="inlineStr">
         <is>
-          <t>Murata Manufacturing / GRM188R72A104KA35D</t>
-        </is>
-      </c>
-      <c r="D7" s="42" t="inlineStr">
-        <is>
-          <t>MLCC / 0.10µF ±10%, 100V, X7R, 0603</t>
+          <t>Northwind Traders</t>
+        </is>
+      </c>
+      <c r="D7" s="43" t="inlineStr">
+        <is>
+          <t>$0.15</t>
         </is>
       </c>
       <c r="E7" s="42" t="inlineStr">
         <is>
-          <t>승인 주품목</t>
+          <t>1개 (Cut Tape)</t>
         </is>
       </c>
       <c r="F7" s="42" t="inlineStr">
         <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="G7" s="42" t="inlineStr">
-        <is>
-          <t>표준 단자 · 현재 CRACK 발생 중. 연성 단자(soft termination) 사양 아님</t>
-        </is>
-      </c>
-      <c r="H7" s="42" t="inlineStr">
-        <is>
-          <t>S-01 · 2026-08-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>대체 후보</t>
+          <t>Litware LW-C0603-104K-100</t>
         </is>
       </c>
       <c r="B8" s="35" t="inlineStr">
         <is>
-          <t>ALT-01</t>
+          <t>0.10µF ±10% 100V X7R 0603</t>
         </is>
       </c>
       <c r="C8" s="35" t="inlineStr">
         <is>
-          <t>KEMET / C0603C104K1RACTU</t>
-        </is>
-      </c>
-      <c r="D8" s="35" t="inlineStr">
-        <is>
-          <t>MLCC / 0.10µF ±10%, 100V, X7R, 0603</t>
+          <t>Northwind Traders</t>
+        </is>
+      </c>
+      <c r="D8" s="44" t="inlineStr">
+        <is>
+          <t>$0.12</t>
         </is>
       </c>
       <c r="E8" s="35" t="inlineStr">
         <is>
-          <t>동급 후보 · 승인 전 사용 금지</t>
+          <t>1개 (Cut Tape)</t>
         </is>
       </c>
       <c r="F8" s="35" t="inlineStr">
         <is>
-          <t>두께·단자·DC-bias·IR·land/reflow</t>
-        </is>
-      </c>
-      <c r="G8" s="35" t="inlineStr">
-        <is>
-          <t>표준 단자 — 굽힘 크랙 완충 없음. 대체해도 개선 근거 없음</t>
-        </is>
-      </c>
-      <c r="H8" s="35" t="inlineStr">
-        <is>
-          <t>S-02 · 2026-08-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>대체 후보</t>
+          <t>Tailspin TS-0603-104M-100</t>
         </is>
       </c>
       <c r="B9" s="35" t="inlineStr">
         <is>
-          <t>ALT-02</t>
+          <t>0.10µF ±20% 100V X7R 0603</t>
         </is>
       </c>
       <c r="C9" s="35" t="inlineStr">
         <is>
-          <t>YAGEO / CC0603KRX7R0BB104</t>
-        </is>
-      </c>
-      <c r="D9" s="35" t="inlineStr">
-        <is>
-          <t>MLCC / 0.10µF, 100V, X7R, 0603 후보</t>
+          <t>Wide World Importers</t>
+        </is>
+      </c>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>$0.09</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>동급 후보 · 승인 전 사용 금지</t>
+          <t>1개 (Cut Tape)</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>두께·단자·DC-bias·IR·land/reflow</t>
-        </is>
-      </c>
-      <c r="G9" s="35" t="inlineStr">
-        <is>
-          <t>표준 단자 — 굽힘 크랙 완충 없음. 대체해도 개선 근거 없음</t>
-        </is>
-      </c>
-      <c r="H9" s="35" t="inlineStr">
-        <is>
-          <t>S-03 · 2026-08-18</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="43" t="inlineStr">
-        <is>
-          <t>단가·MOQ·재고·리드타임·공급사는 이 문서에 싣지 않는다. 조회 시점에 이미 상하는 값이고 품질 담당자의 결정 변수가 아니다 → GET /parts/{part_id} 또는 구매 담당</t>
+      <c r="A11" s="45" t="inlineStr">
+        <is>
+          <t>단가는 데이터시트 기준일의 값이고 발주 근거가 아니다. MOQ·재고·리드타임과 상호호환 판정은 이 문서에 없다 → GET /parts/{part_id} 또는 구매·품질 담당</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0"/>
   <mergeCells count="5">
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <pageMargins left="0.35" right="0.35" top="0.45" bottom="0.45" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
chore: checkpoint workspace before UI improvements
</commit_message>
<xml_diff>
--- a/MAIN_SERVER/templates/불량대책서_샘플_종결본.xlsx
+++ b/MAIN_SERVER/templates/불량대책서_샘플_종결본.xlsx
@@ -30,6 +30,8 @@
     <definedName name="reply_closure_note">'검증'!$B$9</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'대책서'!$A$1:$H$34</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'검증'!$A$1:$H$9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'근거'!$A$1:$E$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'판단자료'!$A$1:$H$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -51,8 +53,9 @@
     </font>
     <font>
       <name val="맑은 고딕"/>
+      <b val="1"/>
       <color rgb="00262626"/>
-      <sz val="9"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
@@ -68,9 +71,8 @@
     </font>
     <font>
       <name val="맑은 고딕"/>
-      <b val="1"/>
       <color rgb="00262626"/>
-      <sz val="8"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
@@ -157,7 +159,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -202,6 +204,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DCE3EF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -281,10 +288,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -292,19 +299,19 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -345,7 +352,7 @@
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -355,15 +362,15 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -376,42 +383,36 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
@@ -500,11 +501,11 @@
   <oneCellAnchor>
     <from>
       <col>0</col>
-      <colOff>276225</colOff>
-      <row>0</row>
-      <rowOff>95250</rowOff>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
     </from>
-    <ext cx="438150" cy="438150"/>
+    <ext cx="5905500" cy="2857500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -512,6 +513,31 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5905500" cy="2857500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -828,7 +854,11 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="1" t="n"/>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CAP</t>
+        </is>
+      </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
           <t>불  량  대  책  서</t>
@@ -929,7 +959,28 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="6" customHeight="1"/>
+    <row r="8" ht="19" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>발행 대상</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Job 7112 · Unit 10412 · CAP-02</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>검사 시각</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-18 16:30:12</t>
+        </is>
+      </c>
+    </row>
     <row r="9" ht="23" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
@@ -1004,12 +1055,12 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>실제 PPM (기준 400)</t>
+          <t>발행 시점 PPM</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>기준 대비</t>
+          <t>발행 기준</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
@@ -1028,8 +1079,10 @@
       <c r="C13" s="13" t="n">
         <v>1280</v>
       </c>
-      <c r="E13" s="14" t="n">
-        <v>3.2</v>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>확정 불량 1건</t>
+        </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
@@ -1040,7 +1093,7 @@
     <row r="14" ht="19" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>발생 집중</t>
+          <t>발생 위치</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -1050,12 +1103,12 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>직전 기간 대비</t>
+          <t>데이터시트 대조</t>
         </is>
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>200 → 1,280 PPM  (6.4배 · 08-18 초과)</t>
+          <t>일치</t>
         </is>
       </c>
     </row>
@@ -1074,10 +1127,7 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>① 발생이 CAP-02·CAP-04에 81.3% 집중(판정 기준 60%) → 부품 Lot보다 공정·설비 원인을 먼저 의심한다.「근거」
-② 최초 초과(08-18)가 mock-v3 적용(08-16)과 3일 이내 → 변경 내용 '그리퍼 파지력 상향 · 배치 하강속도 상향'이 1순위 확인 대상.「판단자료」B
-③ 동일 부품·유형 CLOSED 대책서 1건(2026-04-12 · 배치 하강속도 과다) → 재발. 당시 대책이 왜 듣지 않았는지 먼저 확인한다.「판단자료」C
-④ C-001 대체 후보 2종 · CRACK 관련 소견 2종.「대체품」</t>
+          <t>확정 불량 1건을 기준으로 즉시 발행했다. 발행 시점까지 동일 Job·부품·유형은 16건이며 CAP-02·CAP-04에 13건이 기록됐다. 원인은 자동 추정하지 않으며 담당자가 검사 이미지와 데이터시트 품질 기준을 확인한다.</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1250,7 @@
       <c r="B28" s="20" t="inlineStr">
         <is>
           <t>인라인 AOI 판정 기준이 단자 들뜸과 외관 결손만 보고 있어 미세 굽힘 크랙을 걸러내지 못했다.
-「판단자료」 D 의 MLCC 항목은 '크랙 의심 Lot 단면 또는 비파괴 검사'를 요구하지만, 현재 인라인에는 해당 항목이 없고 단면 검사는 주 1회 샘플로만 돌고 있었다.
+「판단자료」의 MLCC 항목은 '크랙 의심 Lot 단면 또는 비파괴 검사'를 요구하지만, 현재 인라인에는 해당 항목이 없고 단면 검사는 주 1회 샘플로만 돌고 있었다.
 그 결과 08-16 생산분에 이미 크랙이 있었으나 08-18 16:30 임계 초과 시점까지 검출되지 않았다.</t>
         </is>
       </c>
@@ -1251,14 +1301,16 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="37">
+  <mergeCells count="39">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="B26:H27"/>
+    <mergeCell ref="B8:D8"/>
     <mergeCell ref="B1:D3"/>
+    <mergeCell ref="F8:H8"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="A16:A19"/>
     <mergeCell ref="H2:H3"/>
@@ -1294,12 +1346,12 @@
     <dataValidation sqref="F6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="허용되지 않는 값" error="다음 중 하나여야 한다: MISSING,POSITION_ERROR,ORIENTATION_ERROR,CRACK" promptTitle="불량 유형" prompt="별지 3장은 유형과 무관하게 항상 첨부한다.&#10;어느 자료가 이번 건에 쓸모 있는지는 담당자가 판단한다." type="list">
       <formula1>"MISSING,POSITION_ERROR,ORIENTATION_ERROR,CRACK"</formula1>
     </dataValidation>
-    <dataValidation sqref="B21" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="① 협조가 필요한 조치" prompt="담당자 혼자 결정할 수 없는 항목이다. 해당하는 것의 ☐ 를 ☑ 로 바꾸고,&#10;아래 칸에 누구에게 언제 요청했는지 적는다.&#10;&#10;생산 중단 → 생산팀장 · 출하 보류 → 영업/물류 · 재고 선별 → 인력 투입 승인&#10;고객 통보 → 품질보증 책임자 · 설비 정지 → 설비팀&#10;→ containment_summary 첫 줄로 함께 저장된다"/>
-    <dataValidation sqref="B22" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="① 초동 조치 — 오늘 안에" prompt="격리·선별·출하보류 범위와 완료 시각을 적는다.&#10;영향 받는 job_id / unit_id 범위를 함께 적는다.&#10;&#10;원인이 안 나와도 오늘 회신한다. 여기는 '막았는지'만 쓰는 칸이다.&#10;원인을 없애는 것은 ④ 이고, 이 칸은 확산을 멈추는 칸이다.&#10;→ alert_countermeasures.containment_summary"/>
-    <dataValidation sqref="B25" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="② 발생 원인 — 한 줄 요약 (40자)" prompt="아래 본문을 한 줄로 줄인 것. 예: '배치 하강속도 상향 + 지지 핀 최원거리 슬롯'&#10;&#10;이 부품·유형이 다시 나면, 다음 대책서의 자동 분석 ③ 줄이 이 칸을 그대로 읽어&#10;'과거 원인'으로 싣는다. 본문은 길어서 그 자리에 들어가지 않는다.&#10;→ alert_countermeasures.root_cause_label"/>
-    <dataValidation sqref="B26" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="② 발생 원인 — 왜 만들어졌는가" prompt="「판단자료」 A·B로 급증 시점과 레시피 변경 시점을 대조한다.&#10;재현 또는 실물 확인으로 검증한 근거를 적는다.&#10;가설이면 '가설'이라고 표시한다.&#10;→ alert_countermeasures.root_cause_summary"/>
-    <dataValidation sqref="B28" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="③ 유출 원인 — 왜 검사에서 걸리지 않았는가" prompt="「판단자료」 D의 검사 항목과 대조해 판정 기준의 한계를 적는다.&#10;검사를 안 한 것인지, 했는데 못 걸른 것인지 구분한다.&#10;→ alert_countermeasures.escape_cause_summary"/>
-    <dataValidation sqref="B31" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="④ 재발방지 대책 — 원인을 제거하는 영구대책" prompt="레시피·공정조건을 바꾸면 변경 후 recipe_version을 적는다.&#10;부품을 바꾸면 「대체품」 시트의 대체코드를 적는다.&#10;동일 부품을 쓰는 다른 슬롯으로의 수평전개 여부를 포함한다.&#10;&#10;레시피 변경은 변경관리 승인이, 부품 교체는 고객 승인이 필요할 수 있다.&#10;승인 절차가 걸리면 그 일정도 함께 적는다.&#10;→ alert_countermeasures.applied_recipe_version / applied_at"/>
+    <dataValidation sqref="B21" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="① 협조가 필요한 조치" prompt="담당자 혼자 결정할 수 없는 항목이다. 해당하는 것의 ☐ 를 ☑ 로 바꾸고,&#10;아래 칸에 누구에게 언제 요청했는지 적는다.&#10;&#10;생산 중단 → 생산팀장 · 출하 보류 → 영업/물류 · 재고 선별 → 인력 투입 승인&#10;고객 통보 → 품질보증 책임자 · 설비 정지 → 설비팀&#10;"/>
+    <dataValidation sqref="B22" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="① 초동 조치 — 오늘 안에" prompt="격리·선별·출하보류 범위와 완료 시각을 적는다.&#10;영향 받는 job_id / unit_id 범위를 함께 적는다.&#10;&#10;원인이 안 나와도 오늘 회신한다. 여기는 '막았는지'만 쓰는 칸이다.&#10;원인을 없애는 것은 ④ 이고, 이 칸은 확산을 멈추는 칸이다.&#10;"/>
+    <dataValidation sqref="B25" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="② 발생 원인 — 한 줄 요약 (40자)" prompt="아래 본문을 한 줄로 줄인 것. 예: '배치 하강속도 상향 + 지지 핀 최원거리 슬롯'&#10;본문은 길어서 이 칸에 들어가지 않으므로 핵심 원인만 적는다."/>
+    <dataValidation sqref="B26" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="② 발생 원인 — 왜 만들어졌는가" prompt="「근거」의 발생 기록과 검사 이미지를 확인한다.&#10;재현 또는 실물 확인으로 검증한 근거를 적는다.&#10;가설이면 '가설'이라고 표시한다.&#10;"/>
+    <dataValidation sqref="B28" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="③ 유출 원인 — 왜 검사에서 걸리지 않았는가" prompt="「판단자료」의 데이터시트 검사 항목과 대조해 판정 기준의 한계를 적는다.&#10;검사를 안 한 것인지, 했는데 못 걸른 것인지 구분한다.&#10;"/>
+    <dataValidation sqref="B31" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="④ 재발방지 대책 — 원인을 제거하는 영구대책" prompt="레시피·공정조건을 바꾸면 변경 후 recipe_version을 적는다.&#10;부품을 바꾸면 「대체품」 시트의 대체코드를 적는다.&#10;동일 부품을 쓰는 다른 슬롯으로의 수평전개 여부를 포함한다.&#10;&#10;레시피 변경은 변경관리 승인이, 부품 교체는 고객 승인이 필요할 수 있다.&#10;승인 절차가 걸리면 그 일정도 함께 적는다.&#10;"/>
   </dataValidations>
   <pageMargins left="0.35" right="0.35" top="0.45" bottom="0.45" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
@@ -1311,7 +1363,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1493,17 +1544,17 @@
     <mergeCell ref="B4:C4"/>
   </mergeCells>
   <dataValidations count="9">
-    <dataValidation sqref="H5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="허용되지 않는 값" error="다음 중 하나여야 한다: PENDING,EFFECTIVE,INEFFECTIVE" promptTitle="⑤ 판정" prompt="기준 불량률 이하면 EFFECTIVE · 아니면 INEFFECTIVE로 두고 ②로 되돌아간다." type="list">
+    <dataValidation sqref="H5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="허용되지 않는 값" error="다음 중 하나여야 한다: PENDING,EFFECTIVE,INEFFECTIVE" promptTitle="⑤ 판정" prompt="품질 절차에서 정한 판정 기준에 따라 선택한다." type="list">
       <formula1>"PENDING,EFFECTIVE,INEFFECTIVE"</formula1>
     </dataValidation>
-    <dataValidation sqref="B5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 기간" prompt="대책을 적용하고 다시 집계한 구간. [시작, 끝) 으로 적는다.&#10;검증 물량이 기준 최소 건수를 넘어야 판정할 수 있다."/>
-    <dataValidation sqref="D5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 적용 레시피" prompt="대책을 적용한 뒤 실행한 recipe_version.&#10;이 값이 있어야 적용 전후를 같은 제품 안에서 비교할 수 있다.&#10;→ alert_countermeasures.applied_recipe_version"/>
-    <dataValidation sqref="E5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 검사 수량" prompt="부품 기준 검사 건수 (유닛 수 × 해당 부품 슬롯 수).&#10;→ alert_countermeasures.verified_inspected_quantity"/>
-    <dataValidation sqref="F5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 불량 수량" prompt="→ alert_countermeasures.verified_defective_quantity"/>
-    <dataValidation sqref="H5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 판정" prompt="기준 불량률 이하로 내려왔으면 EFFECTIVE.&#10;아니면 INEFFECTIVE로 두고 ②로 되돌아간다.&#10;→ alert_countermeasures.verification_status"/>
-    <dataValidation sqref="B6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 판정 근거" prompt="재집계 결과를 그렇게 읽은 이유.&#10;검증 수량이 기준 최소 건수에 못 미치면 그것도 적는다."/>
-    <dataValidation sqref="F8" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑥ 종결일" prompt="→ alerts.closed_at · alert_status='CLOSED'"/>
-    <dataValidation sqref="B9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑥ 종결 의견" prompt="잔여 위험과 종결 승인 의견.&#10;→ alert_countermeasures.closure_note / closed_by"/>
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 기간" prompt="대책을 적용하고 다시 집계한 구간. [시작, 끝) 으로 적는다.&#10;"/>
+    <dataValidation sqref="D5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 적용 레시피" prompt="대책을 적용한 뒤 실행한 recipe_version.&#10;이 값이 있어야 적용 전후를 같은 제품 안에서 비교할 수 있다.&#10;"/>
+    <dataValidation sqref="E5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 검사 수량" prompt="부품 기준 검사 건수 (유닛 수 × 해당 부품 슬롯 수).&#10;"/>
+    <dataValidation sqref="F5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 불량 수량" prompt=""/>
+    <dataValidation sqref="H5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 판정" prompt="판정 기준과 비교한 결론을 선택한다.&#10;기준은 해당 품질 절차에서 확인한다."/>
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 판정 근거" prompt="재집계 결과를 그렇게 읽은 이유.&#10;"/>
+    <dataValidation sqref="F8" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑥ 종결일" prompt=""/>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑥ 종결 의견" prompt="잔여 위험과 종결 승인 의견.&#10;"/>
   </dataValidations>
   <pageMargins left="0.35" right="0.35" top="0.45" bottom="0.45" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -1516,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1816,21 +1867,47 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>검사 이미지</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>샘플 이미지 미포함 · InspectionSamples/mock-fail.jpg · SHA-256 —</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="34" t="n"/>
+    </row>
+    <row r="22" ht="40" customHeight="1"/>
+    <row r="23" ht="40" customHeight="1"/>
+    <row r="24" ht="40" customHeight="1"/>
+    <row r="25" ht="40" customHeight="1"/>
+    <row r="26" ht="40" customHeight="1"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0"/>
-  <mergeCells count="9">
+  <mergeCells count="12">
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="D5:E5"/>
+    <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="A21:E26"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.35" right="0.35" top="0.45" bottom="0.45" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1840,586 +1917,134 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>판단 자료</t>
+          <t>품질 기준        [조회 시점 참조]</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="27" t="inlineStr">
         <is>
-          <t>담당자가 ②발생 원인 · ③유출 원인을 좁히는 데 쓰는 참고 자료 · 자동 조회 · 결재 대상 아님</t>
+          <t>부품 데이터시트 Checklist 시트에서 조회 · 원인 자동 추정 자료가 아님</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="33" t="inlineStr">
-        <is>
-          <t>판단 순서    ①「근거」어느 슬롯에 몰렸나  →  ② A 언제부터 올랐나  →  ③ B 그때 무엇이 바뀌었나  →  ④ C 전에도 있었나  →  ⑤ D 무엇을 확인하나</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17" customHeight="1">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>부품 범주 MLCC · 데이터시트 대조 일치 · 기준일 2026-08-18 · 조회 2026-08-19 09:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="28" t="inlineStr">
         <is>
-          <t>A.  주차별 추세        [발행 시점 고정]</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="14" customHeight="1">
-      <c r="A6" s="27" t="inlineStr">
-        <is>
-          <t>언제부터 올라갔는지 · 급변 시점과 아래 B의 레시피 변경 시점을 대조한다. 주차 경계와 대책서 집계 구간은 일치하지 않는다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="29" t="inlineStr">
-        <is>
-          <t>주차</t>
-        </is>
-      </c>
-      <c r="B7" s="29" t="inlineStr">
-        <is>
-          <t>검사 수량</t>
-        </is>
-      </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>불량 수량</t>
-        </is>
-      </c>
-      <c r="D7" s="29" t="inlineStr">
-        <is>
-          <t>불량률</t>
-        </is>
-      </c>
-      <c r="E7" s="29" t="inlineStr">
-        <is>
-          <t>기준 대비</t>
-        </is>
-      </c>
-      <c r="F7" s="29" t="inlineStr">
-        <is>
-          <t>레시피</t>
-        </is>
-      </c>
-      <c r="G7" s="29" t="inlineStr">
-        <is>
-          <t>비고</t>
-        </is>
-      </c>
-      <c r="H7" s="30" t="n"/>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>2026-W29</t>
-        </is>
-      </c>
-      <c r="B8" s="31" t="n">
-        <v>12400</v>
-      </c>
-      <c r="C8" s="31" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="26" t="n">
-        <v>0.0001612903225806452</v>
-      </c>
-      <c r="E8" s="34" t="n">
-        <v>0.4032258064516129</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>mock-v1</t>
-        </is>
-      </c>
-      <c r="G8" s="32" t="n"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>2026-W30</t>
-        </is>
-      </c>
-      <c r="B9" s="31" t="n">
-        <v>12550</v>
-      </c>
-      <c r="C9" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" s="26" t="n">
-        <v>0.0002390438247011952</v>
-      </c>
-      <c r="E9" s="34" t="n">
-        <v>0.5976095617529881</v>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>mock-v1</t>
-        </is>
-      </c>
-      <c r="G9" s="32" t="n"/>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>2026-W31</t>
-        </is>
-      </c>
-      <c r="B10" s="31" t="n">
-        <v>12480</v>
-      </c>
-      <c r="C10" s="31" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="26" t="n">
-        <v>0.0001602564102564103</v>
-      </c>
-      <c r="E10" s="34" t="n">
-        <v>0.4006410256410256</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>mock-v2</t>
-        </is>
-      </c>
-      <c r="G10" s="32" t="inlineStr">
-        <is>
-          <t>08-05 mock-v2 적용</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>2026-W32</t>
-        </is>
-      </c>
-      <c r="B11" s="31" t="n">
-        <v>12575</v>
-      </c>
-      <c r="C11" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="26" t="n">
-        <v>0.0002385685884691849</v>
-      </c>
-      <c r="E11" s="34" t="n">
-        <v>0.5964214711729622</v>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>mock-v2</t>
-        </is>
-      </c>
-      <c r="G11" s="32" t="n"/>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>2026-W33</t>
-        </is>
-      </c>
-      <c r="B12" s="31" t="n">
-        <v>12650</v>
-      </c>
-      <c r="C12" s="31" t="n">
-        <v>8</v>
-      </c>
-      <c r="D12" s="26" t="n">
-        <v>0.0006324110671936759</v>
-      </c>
-      <c r="E12" s="34" t="n">
-        <v>1.58102766798419</v>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>mock-v3</t>
-        </is>
-      </c>
-      <c r="G12" s="32" t="inlineStr">
-        <is>
-          <t>08-16 mock-v3 적용 · 급증 시점</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>2026-W34</t>
-        </is>
-      </c>
-      <c r="B13" s="31" t="n">
-        <v>5420</v>
-      </c>
-      <c r="C13" s="31" t="n">
-        <v>8</v>
-      </c>
-      <c r="D13" s="26" t="n">
-        <v>0.001476014760147601</v>
-      </c>
-      <c r="E13" s="34" t="n">
-        <v>3.690036900369003</v>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>mock-v3</t>
-        </is>
-      </c>
-      <c r="G13" s="32" t="inlineStr">
-        <is>
-          <t>진행 중 · 08-19 09:00 기준</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="28" t="inlineStr">
-        <is>
-          <t>B.  레시피 변경 전후 불량률        [발행 시점 고정]</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="14" customHeight="1">
-      <c r="A16" s="27" t="inlineStr">
-        <is>
-          <t>datastation_part_rates · 공정 조건이 원인인지 부품이 원인인지 가르는 1차 근거</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="29" t="inlineStr">
-        <is>
-          <t>레시피</t>
-        </is>
-      </c>
-      <c r="B17" s="29" t="inlineStr">
-        <is>
-          <t>적용 기간</t>
-        </is>
-      </c>
-      <c r="C17" s="29" t="inlineStr">
-        <is>
-          <t>검사 수량</t>
-        </is>
-      </c>
-      <c r="D17" s="29" t="inlineStr">
-        <is>
-          <t>불량 수량</t>
-        </is>
-      </c>
-      <c r="E17" s="29" t="inlineStr">
-        <is>
-          <t>불량률</t>
-        </is>
-      </c>
-      <c r="F17" s="29" t="inlineStr">
-        <is>
-          <t>기준 대비</t>
-        </is>
-      </c>
-      <c r="G17" s="29" t="inlineStr">
-        <is>
-          <t>변경 내용</t>
-        </is>
-      </c>
-      <c r="H17" s="30" t="n"/>
-    </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>mock-v1</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>~ 2026-08-05</t>
-        </is>
-      </c>
-      <c r="C18" s="31" t="n">
-        <v>124000</v>
-      </c>
-      <c r="D18" s="31" t="n">
-        <v>20</v>
-      </c>
-      <c r="E18" s="26" t="n">
-        <v>0.0001612903225806452</v>
-      </c>
-      <c r="F18" s="34" t="n">
-        <v>0.4032258064516129</v>
-      </c>
-      <c r="G18" s="35" t="inlineStr">
-        <is>
-          <t>기준 레시피</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>mock-v2</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>08-05 ~ 08-16</t>
-        </is>
-      </c>
-      <c r="C19" s="31" t="n">
-        <v>99500</v>
-      </c>
-      <c r="D19" s="31" t="n">
-        <v>24</v>
-      </c>
-      <c r="E19" s="26" t="n">
-        <v>0.0002412060301507538</v>
-      </c>
-      <c r="F19" s="34" t="n">
-        <v>0.6030150753768844</v>
-      </c>
-      <c r="G19" s="35" t="inlineStr">
-        <is>
-          <t>픽업 속도 조정</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>mock-v3</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>08-16 ~ 현재</t>
-        </is>
-      </c>
-      <c r="C20" s="31" t="n">
-        <v>30600</v>
-      </c>
-      <c r="D20" s="31" t="n">
-        <v>33</v>
-      </c>
-      <c r="E20" s="26" t="n">
-        <v>0.00107843137254902</v>
-      </c>
-      <c r="F20" s="34" t="n">
-        <v>2.696078431372549</v>
-      </c>
-      <c r="G20" s="35" t="inlineStr">
-        <is>
-          <t>그리퍼 파지력 상향 · 배치 하강속도 상향 — 변경 직후 CRACK 급증</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="28" t="inlineStr">
-        <is>
-          <t>C.  동일 부품 · 동일 유형 과거 대책서        [발행 시점 고정]</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="14" customHeight="1">
-      <c r="A23" s="27" t="inlineStr">
-        <is>
-          <t>datastation_alerts · 재발이면 이전 대책이 왜 듣지 않았는지부터 확인한다</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="29" t="inlineStr">
-        <is>
-          <t>문서번호</t>
-        </is>
-      </c>
-      <c r="B24" s="29" t="inlineStr">
-        <is>
-          <t>집계 기간</t>
-        </is>
-      </c>
-      <c r="C24" s="29" t="inlineStr">
-        <is>
-          <t>불량률</t>
-        </is>
-      </c>
-      <c r="D24" s="29" t="inlineStr">
-        <is>
-          <t>상태</t>
-        </is>
-      </c>
-      <c r="E24" s="29" t="inlineStr">
-        <is>
-          <t>적용 대책</t>
-        </is>
-      </c>
-      <c r="F24" s="30" t="n"/>
-      <c r="G24" s="29" t="inlineStr">
-        <is>
-          <t>당시 근본 원인</t>
-        </is>
-      </c>
-      <c r="H24" s="30" t="n"/>
-    </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="36" t="inlineStr">
-        <is>
-          <t>QA-CAP-CRACK-20260412-001</t>
-        </is>
-      </c>
-      <c r="B25" s="36" t="inlineStr">
-        <is>
-          <t>2026-04-05 ~ 04-12</t>
-        </is>
-      </c>
-      <c r="C25" s="37" t="n">
-        <v>0.0009</v>
-      </c>
-      <c r="D25" s="36" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="E25" s="38" t="inlineStr">
-        <is>
-          <t>mock-v1 / 04-15</t>
-        </is>
-      </c>
-      <c r="G25" s="35" t="inlineStr">
-        <is>
-          <t>배치 하강속도 과다로 착지 충격. 속도 하향 후 160 PPM으로 회복.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="17" customHeight="1">
-      <c r="A27" s="28" t="inlineStr">
-        <is>
-          <t>D.  품질 체크리스트        [조회 시점 참조 · 데이터시트 갱신 시 바뀜]</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="14" customHeight="1">
-      <c r="A28" s="27" t="inlineStr">
-        <is>
-          <t>데이터시트 Checklist 시트 · 범주 = part_groups.category_label · 이 범주에서 무엇을 확인해야 하는지</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="29" t="inlineStr">
+          <t>데이터시트 품질 체크리스트</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B29" s="29" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>확인 항목</t>
         </is>
       </c>
-      <c r="C29" s="39" t="n"/>
-      <c r="D29" s="30" t="n"/>
-      <c r="E29" s="29" t="inlineStr">
+      <c r="C6" s="36" t="n"/>
+      <c r="D6" s="30" t="n"/>
+      <c r="E6" s="29" t="inlineStr">
         <is>
           <t>이상 시 조치</t>
         </is>
       </c>
-      <c r="F29" s="39" t="n"/>
-      <c r="G29" s="39" t="n"/>
-      <c r="H29" s="30" t="n"/>
-    </row>
-    <row r="30" ht="40" customHeight="1">
-      <c r="A30" s="40" t="inlineStr">
+      <c r="F6" s="36" t="n"/>
+      <c r="G6" s="36" t="n"/>
+      <c r="H6" s="30" t="n"/>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t>입고 검사</t>
         </is>
       </c>
-      <c r="B30" s="35" t="inlineStr">
+      <c r="B7" s="38" t="inlineStr">
         <is>
           <t>외관/단자, 0603·100V·X7R 확인, LCR·절연저항 샘플</t>
         </is>
       </c>
-      <c r="E30" s="35" t="inlineStr">
+      <c r="E7" s="38" t="inlineStr">
         <is>
           <t>크랙/IR 저하는 Lot·패널 위치별 격리, 보드 굴곡·분리·프로브 지지 조건을 재현하고 공정 조건 수정</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="40" customHeight="1">
-      <c r="A31" s="40" t="inlineStr">
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t>조립·보관</t>
         </is>
       </c>
-      <c r="B31" s="35" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>land/reflow 준수; panel depanel·ICT probe·connector 체결 시 board support로 보드 굽힘 억제</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="40" customHeight="1">
-      <c r="A32" s="40" t="inlineStr">
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>기능·신뢰성</t>
         </is>
       </c>
-      <c r="B32" s="35" t="inlineStr">
+      <c r="B9" s="38" t="inlineStr">
         <is>
           <t>AOI, LCR/IR; crack 의심 Lot 단면 또는 비파괴 검사</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>원본 semiconductor_assembly_quality_datasheet_2026-08-18.xlsx</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0"/>
-  <mergeCells count="32">
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="E30:H32"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="G11:H11"/>
+  <mergeCells count="11">
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="A27:H27"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="E7:H9"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="E29:H29"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A11:H11"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B6:D6"/>
   </mergeCells>
   <pageMargins left="0.35" right="0.35" top="0.45" bottom="0.45" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2429,7 +2054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2443,163 +2068,195 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>대체품 후보        [조회 시점 참조]</t>
+          <t>현재 부품과 대체품 후보        [조회 시점 참조]</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="27" t="inlineStr">
         <is>
-          <t>불량 유형과 무관하게 항상 첨부한다 · 부품 교체가 이번 건의 대책인지는 ② 발생 원인을 확정한 담당자가 판단한다</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="41" t="inlineStr">
+          <t>DB parts: CAP / Contoso CX-0603X7R104K100 / MLCC · 데이터시트 MPN 대조: 일치</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>현재 MPN</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>핵심 정격</t>
+        </is>
+      </c>
+      <c r="C3" s="29" t="inlineStr">
+        <is>
+          <t>공급사</t>
+        </is>
+      </c>
+      <c r="D3" s="29" t="inlineStr">
+        <is>
+          <t>단가</t>
+        </is>
+      </c>
+      <c r="E3" s="29" t="inlineStr">
+        <is>
+          <t>가격 기준 수량</t>
+        </is>
+      </c>
+      <c r="F3" s="29" t="inlineStr">
+        <is>
+          <t>가격 확인일</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="39" t="inlineStr">
+        <is>
+          <t>Contoso CX-0603X7R104K100</t>
+        </is>
+      </c>
+      <c r="B4" s="39" t="inlineStr">
+        <is>
+          <t>0.10µF ±10% 100V X7R 0603</t>
+        </is>
+      </c>
+      <c r="C4" s="39" t="inlineStr">
+        <is>
+          <t>Northwind Traders</t>
+        </is>
+      </c>
+      <c r="D4" s="40" t="inlineStr">
+        <is>
+          <t>$0.15</t>
+        </is>
+      </c>
+      <c r="E4" s="39" t="inlineStr">
+        <is>
+          <t>1개 (Cut Tape)</t>
+        </is>
+      </c>
+      <c r="F4" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="41" t="inlineStr">
         <is>
           <t>같은 부품 타입이라는 것 외에 검증된 것은 없다 · 동일 정격만으로 drop-in 판단 금지 · 핀/패키지/정격/열/수명 재검증과 변경 승인을 거친 뒤에만 적용한다.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="23" t="inlineStr">
-        <is>
-          <t>조회 시각 2026-08-19 09:00:00   ·   데이터시트 semiconductor_assembly_quality_datasheet_2026-08-18.xlsx (기준일 2026-08-18)   ·   부품 타입 MLCC   ·   후보 3종   ·   단가 $0.09 ~ $0.15   ·   현재 선정 $0.15</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="29" t="inlineStr">
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>조회 시각 2026-08-19 09:00:00   ·   데이터시트 semiconductor_assembly_quality_datasheet_2026-08-18.xlsx (기준일 2026-08-18)   ·   부품 타입 MLCC   ·   후보 2종   ·   단가 $0.09 ~ $0.15   ·   현재 선정 $0.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>제조사 / P/N</t>
         </is>
       </c>
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>핵심 정격</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C9" s="29" t="inlineStr">
         <is>
           <t>공급사</t>
         </is>
       </c>
-      <c r="D6" s="29" t="inlineStr">
+      <c r="D9" s="29" t="inlineStr">
         <is>
           <t>단가</t>
         </is>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E9" s="29" t="inlineStr">
         <is>
           <t>가격 기준 수량</t>
         </is>
       </c>
-      <c r="F6" s="29" t="inlineStr">
+      <c r="F9" s="29" t="inlineStr">
         <is>
           <t>가격 확인일</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1">
-      <c r="A7" s="42" t="inlineStr">
-        <is>
-          <t>Contoso CX-0603X7R104K100</t>
-        </is>
-      </c>
-      <c r="B7" s="42" t="inlineStr">
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="38" t="inlineStr">
+        <is>
+          <t>Litware LW-C0603-104K-100</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>0.10µF ±10% 100V X7R 0603</t>
         </is>
       </c>
-      <c r="C7" s="42" t="inlineStr">
+      <c r="C10" s="38" t="inlineStr">
         <is>
           <t>Northwind Traders</t>
         </is>
       </c>
-      <c r="D7" s="43" t="inlineStr">
-        <is>
-          <t>$0.15</t>
-        </is>
-      </c>
-      <c r="E7" s="42" t="inlineStr">
+      <c r="D10" s="42" t="inlineStr">
+        <is>
+          <t>$0.12</t>
+        </is>
+      </c>
+      <c r="E10" s="38" t="inlineStr">
         <is>
           <t>1개 (Cut Tape)</t>
         </is>
       </c>
-      <c r="F7" s="42" t="inlineStr">
+      <c r="F10" s="38" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="54" customHeight="1">
-      <c r="A8" s="35" t="inlineStr">
-        <is>
-          <t>Litware LW-C0603-104K-100</t>
-        </is>
-      </c>
-      <c r="B8" s="35" t="inlineStr">
-        <is>
-          <t>0.10µF ±10% 100V X7R 0603</t>
-        </is>
-      </c>
-      <c r="C8" s="35" t="inlineStr">
-        <is>
-          <t>Northwind Traders</t>
-        </is>
-      </c>
-      <c r="D8" s="44" t="inlineStr">
-        <is>
-          <t>$0.12</t>
-        </is>
-      </c>
-      <c r="E8" s="35" t="inlineStr">
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="38" t="inlineStr">
+        <is>
+          <t>Tailspin TS-0603-104M-100</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>0.10µF ±20% 100V X7R 0603</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="inlineStr">
+        <is>
+          <t>Wide World Importers</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>$0.09</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
         <is>
           <t>1개 (Cut Tape)</t>
         </is>
       </c>
-      <c r="F8" s="35" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="54" customHeight="1">
-      <c r="A9" s="35" t="inlineStr">
-        <is>
-          <t>Tailspin TS-0603-104M-100</t>
-        </is>
-      </c>
-      <c r="B9" s="35" t="inlineStr">
-        <is>
-          <t>0.10µF ±20% 100V X7R 0603</t>
-        </is>
-      </c>
-      <c r="C9" s="35" t="inlineStr">
-        <is>
-          <t>Wide World Importers</t>
-        </is>
-      </c>
-      <c r="D9" s="44" t="inlineStr">
-        <is>
-          <t>$0.09</t>
-        </is>
-      </c>
-      <c r="E9" s="35" t="inlineStr">
-        <is>
-          <t>1개 (Cut Tape)</t>
-        </is>
-      </c>
-      <c r="F9" s="35" t="inlineStr">
+      <c r="F11" s="38" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="45" t="inlineStr">
-        <is>
-          <t>단가는 데이터시트 기준일의 값이고 발주 근거가 아니다. MOQ·재고·리드타임과 상호호환 판정은 이 문서에 없다 → GET /parts/{part_id} 또는 구매·품질 담당</t>
+    <row r="13">
+      <c r="A13" s="43" t="inlineStr">
+        <is>
+          <t>단가는 데이터시트 기준일의 값이고 발주 근거가 아니다. MOQ·재고·리드타임과 상호호환 판정은 이 문서에 없다 → GET /parts/CAP 또는 구매·품질 담당</t>
         </is>
       </c>
     </row>
@@ -2607,10 +2264,10 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0"/>
   <mergeCells count="5">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <pageMargins left="0.35" right="0.35" top="0.45" bottom="0.45" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
chore: checkpoint current workspace state
</commit_message>
<xml_diff>
--- a/MAIN_SERVER/templates/불량대책서_샘플_종결본.xlsx
+++ b/MAIN_SERVER/templates/불량대책서_샘플_종결본.xlsx
@@ -43,7 +43,7 @@
     <numFmt numFmtId="164" formatCode="0.0&quot;배&quot;"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -106,7 +106,7 @@
     <font>
       <name val="맑은 고딕"/>
       <color rgb="00262626"/>
-      <sz val="8.5"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
@@ -123,11 +123,6 @@
       <name val="맑은 고딕"/>
       <b val="1"/>
       <color rgb="00808080"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <color rgb="00262626"/>
       <sz val="8"/>
     </font>
     <font>
@@ -336,7 +331,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -348,7 +343,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -356,10 +351,10 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -373,36 +368,36 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -411,13 +406,13 @@
     <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -1090,7 +1085,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="19" customHeight="1">
+    <row r="14" ht="34" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>발생 위치</t>
@@ -1103,12 +1098,13 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>데이터시트 대조</t>
+          <t>제조사 P/N</t>
         </is>
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>일치</t>
+          <t>일치 · Contoso CX-0603X7R104K100
+정격 0.10µF ±10% 100V X7R 0603 · 공급사 Northwind Traders</t>
         </is>
       </c>
     </row>

</xml_diff>